<commit_message>
Realizacion de ejercicio semana 2
</commit_message>
<xml_diff>
--- a/Semana 2/inventario.xlsx
+++ b/Semana 2/inventario.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,7 +424,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>producto</t>
+          <t>nombre</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -439,17 +439,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>precio_compra</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>precio_venta</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>proveedor</t>
+          <t>precio</t>
         </is>
       </c>
     </row>
@@ -459,27 +449,19 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Teclado</t>
+          <t>Notebook</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Periférico</t>
+          <t>Electrónica</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="E2" t="n">
-        <v>8000</v>
-      </c>
-      <c r="F2" t="n">
-        <v>15000</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>TechCorp</t>
-        </is>
+        <v>1200</v>
       </c>
     </row>
     <row r="3">
@@ -493,22 +475,14 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Periférico</t>
+          <t>Accesorios</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="E3" t="n">
-        <v>4000</v>
-      </c>
-      <c r="F3" t="n">
-        <v>8000</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>TechCorp</t>
-        </is>
+        <v>25</v>
       </c>
     </row>
     <row r="4">
@@ -517,27 +491,19 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Teclado</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Pantalla</t>
+          <t>Accesorios</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="E4" t="n">
-        <v>80000</v>
-      </c>
-      <c r="F4" t="n">
-        <v>120000</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>DisplaySA</t>
-        </is>
+        <v>45</v>
       </c>
     </row>
     <row r="5">
@@ -546,201 +512,19 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Notebook</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Computadora</t>
+          <t>Electrónica</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E5" t="n">
-        <v>300000</v>
-      </c>
-      <c r="F5" t="n">
-        <v>450000</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>CompuMundo</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Auriculares</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Audio</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>60</v>
-      </c>
-      <c r="E6" t="n">
-        <v>4000</v>
-      </c>
-      <c r="F6" t="n">
-        <v>7000</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>SoundPro</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Webcam</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Video</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>30</v>
-      </c>
-      <c r="E7" t="n">
-        <v>8000</v>
-      </c>
-      <c r="F7" t="n">
-        <v>15000</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>VisionTech</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Parlantes</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Audio</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>25</v>
-      </c>
-      <c r="E8" t="n">
-        <v>12000</v>
-      </c>
-      <c r="F8" t="n">
-        <v>20000</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>SoundPro</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Impresora</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Oficina</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>15</v>
-      </c>
-      <c r="E9" t="n">
-        <v>50000</v>
-      </c>
-      <c r="F9" t="n">
-        <v>80000</v>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>PrintMax</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Tablet</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Dispositivo</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>18</v>
-      </c>
-      <c r="E10" t="n">
-        <v>60000</v>
-      </c>
-      <c r="F10" t="n">
-        <v>90000</v>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>MobileTech</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Disco SSD</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Almacenamiento</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>40</v>
-      </c>
-      <c r="E11" t="n">
-        <v>35000</v>
-      </c>
-      <c r="F11" t="n">
-        <v>60000</v>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>StoragePlus</t>
-        </is>
+        <v>300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>